<commit_message>
+Create shop panel for Rare, Promotion and Bundle.
</commit_message>
<xml_diff>
--- a/Tool/data/Shop.xlsx
+++ b/Tool/data/Shop.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="72">
   <si>
     <t>ProductID</t>
   </si>
@@ -176,7 +176,7 @@
     <t>rare_exp</t>
   </si>
   <si>
-    <t>ZhuBajie_avatar</t>
+    <t>ZhuBaJie</t>
   </si>
   <si>
     <t>supreme_exp</t>
@@ -1159,7 +1159,7 @@
         <v>100</v>
       </c>
       <c r="J14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K14" t="s">
         <v>65</v>
@@ -1206,7 +1206,7 @@
         <v>120</v>
       </c>
       <c r="J15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K15" t="s">
         <v>65</v>
@@ -1253,7 +1253,7 @@
         <v>8000</v>
       </c>
       <c r="J16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K16" t="s">
         <v>65</v>
@@ -1300,7 +1300,7 @@
         <v>10000</v>
       </c>
       <c r="J17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K17" t="s">
         <v>65</v>
@@ -1489,7 +1489,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1527,54 +1527,54 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
         <v>55</v>
       </c>
       <c r="C5">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C6">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C7">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C8">
         <v>10</v>
@@ -1582,13 +1582,79 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
         <v>59</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>59</v>
+      </c>
+      <c r="B14" t="s">
         <v>45</v>
       </c>
-      <c r="C9">
+      <c r="C14">
         <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>